<commit_message>
bug fix: 1. merge the tables into the same file for announcement scraper 2. modify the format of pdf_parser
</commit_message>
<xml_diff>
--- a/downloads/2454_2026_Q1_重大有價證券.xlsx
+++ b/downloads/2454_2026_Q1_重大有價證券.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,7 +480,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>持股比例</t>
+          <t>持股</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -495,71 +495,55 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>強制透過損益按公允價值衡量之金融資產－流動</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>組合式商品</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>JPMorgan Chase &amp; Co.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>旭展(香港)投資有限公司</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>股數</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>USD 17,737</t>
+          <t>帳面金額</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>比例</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>USD 17,737</t>
+          <t>公允價值</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>備註</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>強制透過損益按公允價值衡量之金融資產－非流動</t>
+          <t>強制透過損益按公允價值衡量之金融資產－流動</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>信託基金</t>
+          <t>組合式商品</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>信託基金</t>
+          <t>JPMorgan Chase &amp; Co.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MediaTek USA Inc.</t>
+          <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -569,7 +553,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>USD 85,438</t>
+          <t>USD 17,737</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -579,7 +563,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>USD 85,438</t>
+          <t>USD 17,737</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -596,17 +580,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>債券</t>
+          <t>信託基金</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Carsome Group Convertible Promissory Note</t>
+          <t>信託基金</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MTKC Global Holdings Co. Limited</t>
+          <t>MediaTek USA Inc.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -616,7 +600,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>USD 12,830</t>
+          <t>USD 85,438</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -626,7 +610,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>USD 12,830</t>
+          <t>USD 85,438</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -638,7 +622,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>透過其他綜合損益按公允價值衡量之債務工具－流動</t>
+          <t>強制透過損益按公允價值衡量之金融資產－非流動</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -648,12 +632,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
+          <t>Carsome Group Convertible Promissory Note</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>旭展(香港)投資有限公司</t>
+          <t>MTKC Global Holdings Co. Limited</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -663,7 +647,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>USD 19,810</t>
+          <t>USD 12,830</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -673,7 +657,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>USD 19,810</t>
+          <t>USD 12,830</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -685,42 +669,42 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>透過其他綜合損益按公允價值衡量之權益工具－流動</t>
+          <t>透過其他綜合損益按公允價值衡量之債務工具－流動</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>股票</t>
+          <t>債券</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>深圳市匯頂科技股份有限公司</t>
+          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>匯發國際(香港)有限公司</t>
+          <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>12,476,705</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>USD 114,441</t>
+          <t>USD 19,810</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3 %</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>USD 114,441</t>
+          <t>USD 19,810</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -742,32 +726,32 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>晶心科技(股)公司</t>
+          <t>深圳市匯頂科技股份有限公司</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>翔發投資(股)公司</t>
+          <t>匯發國際(香港)有限公司</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3,249,324</t>
+          <t>12,476,705</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>$ 558,884</t>
+          <t>USD 114,441</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6 %</t>
+          <t>3 %</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>$ 558,884</t>
+          <t>USD 114,441</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -789,7 +773,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>中華精測科技(股)公司</t>
+          <t>晶心科技(股)公司</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -799,22 +783,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>176,000</t>
+          <t>3,249,324</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>$ 542,080</t>
+          <t>$ 558,884</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1 %</t>
+          <t>6 %</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>$ 542,080</t>
+          <t>$ 558,884</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -826,7 +810,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
+          <t>透過其他綜合損益按公允價值衡量之權益工具－流動</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -836,32 +820,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>富邦金融控股(股)公司乙種特別股</t>
+          <t>中華精測科技(股)公司</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>翔發投資(股)公司</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15,000,000</t>
+          <t>176,000</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>$ 937,500</t>
+          <t>$ 542,080</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>$ 937,500</t>
+          <t>$ 542,080</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -883,7 +867,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>富邦金融控股(股)公司丙種特別股</t>
+          <t>富邦金融控股(股)公司乙種特別股</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -893,12 +877,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>7,056,243</t>
+          <t>15,000,000</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>$ 364,102</t>
+          <t>$ 937,500</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -908,7 +892,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>$ 364,102</t>
+          <t>$ 937,500</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -930,32 +914,32 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>深圳傳音控股股份有限公司</t>
+          <t>富邦金融控股(股)公司丙種特別股</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Digimoc Holdings Limited</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>71,573,109</t>
+          <t>7,056,243</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>USD 568,139</t>
+          <t>$ 364,102</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>6 %</t>
+          <t>0 %</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>USD 568,139</t>
+          <t>$ 364,102</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -977,7 +961,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AutoX, Inc.</t>
+          <t>深圳傳音控股股份有限公司</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -987,22 +971,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>55,009,500</t>
+          <t>71,573,109</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>USD 80,864</t>
+          <t>USD 568,139</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3 %</t>
+          <t>6 %</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>USD 80,864</t>
+          <t>USD 568,139</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1024,7 +1008,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Aeonsemi, Inc.</t>
+          <t>AutoX, Inc.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1034,22 +1018,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1,417,657</t>
+          <t>55,009,500</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>USD 18,592</t>
+          <t>USD 80,864</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6 %</t>
+          <t>3 %</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>USD 18,592</t>
+          <t>USD 80,864</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1071,32 +1055,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>世芯電子股份有限公司</t>
+          <t>Aeonsemi, Inc.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>聯發資本(股)公司</t>
+          <t>Digimoc Holdings Limited</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>450,000</t>
+          <t>1,417,657</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>$ 991,809</t>
+          <t>USD 18,592</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1 %</t>
+          <t>6 %</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>$ 991,809</t>
+          <t>USD 18,592</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1118,32 +1102,32 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ITH Corporation</t>
+          <t>世芯電子股份有限公司</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Gaintech Co. Limited</t>
+          <t>聯發資本(股)公司</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>53,889,085</t>
+          <t>450,000</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>USD 55,098</t>
+          <t>$ 991,809</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>11 %</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>USD 55,098</t>
+          <t>$ 991,809</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1165,32 +1149,32 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TRANSSNET TECHNOLOGY INC.</t>
+          <t>ITH Corporation</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Cloud Ranger Limited</t>
+          <t>Gaintech Co. Limited</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1,970,316</t>
+          <t>53,889,085</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>USD 10,730</t>
+          <t>USD 55,098</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>11 %</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>USD 10,730</t>
+          <t>USD 55,098</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1212,7 +1196,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Scaleflux Inc.</t>
+          <t>TRANSSNET TECHNOLOGY INC.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1222,22 +1206,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2,096,587</t>
+          <t>1,970,316</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>USD 17,475</t>
+          <t>USD 10,730</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2 %</t>
+          <t>8 %</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>USD 17,475</t>
+          <t>USD 10,730</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1259,32 +1243,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>瀚博半導體(上海)有限公司</t>
+          <t>Scaleflux Inc.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MTKC Global Holdings Co. Limited</t>
+          <t>Cloud Ranger Limited</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4,252,861</t>
+          <t>2,096,587</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>USD 37,420</t>
+          <t>USD 17,475</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>1 %</t>
+          <t>2 %</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>USD 37,420</t>
+          <t>USD 17,475</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1306,32 +1290,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>強一半導體(蘇州)有限公司</t>
+          <t>瀚博半導體(上海)有限公司</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>聯發利寶(香港)有限公司</t>
+          <t>MTKC Global Holdings Co. Limited</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2,474,300</t>
+          <t>4,252,861</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>CNY 586,409</t>
+          <t>USD 37,420</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2 %</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CNY 586,409</t>
+          <t>USD 37,420</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1353,32 +1337,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>蘇州思必馳信息科技有限公司</t>
+          <t>強一半導體(蘇州)有限公司</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>聯發博動科技(北京)有限公司</t>
+          <t>聯發利寶(香港)有限公司</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4,638,600</t>
+          <t>2,474,300</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CNY 75,907</t>
+          <t>CNY 586,409</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>1 %</t>
+          <t>2 %</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CNY 75,907</t>
+          <t>CNY 586,409</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1400,37 +1384,37 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>蘇州思必馳信息科技有限公司</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>翔發投資(股)公司</t>
+          <t>聯發博動科技(北京)有限公司</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>7,794,085</t>
+          <t>4,638,600</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>$ 11,613,187</t>
+          <t>CNY 75,907</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>$ 11,613,187</t>
+          <t>CNY 75,907</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>註1</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1431,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>樺漢科技股份有限公司</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1457,27 +1441,27 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3,682,456</t>
+          <t>7,794,085</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>$ 997,946</t>
+          <t>$ 11,613,187</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>3 %</t>
+          <t>0 %</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>$ 997,946</t>
+          <t>$ 11,613,187</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>註1</t>
         </is>
       </c>
     </row>
@@ -1494,32 +1478,32 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>欣興電子股份有限公司</t>
+          <t>樺漢科技股份有限公司</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>聯發資本(股)公司</t>
+          <t>翔發投資(股)公司</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>800,000</t>
+          <t>3,682,456</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>$ 355,600</t>
+          <t>$ 997,946</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>3 %</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>$ 355,600</t>
+          <t>$ 997,946</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1541,32 +1525,32 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Ayar Labs, Inc.</t>
+          <t>欣興電子股份有限公司</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Digimoc Holdings Limited</t>
+          <t>聯發資本(股)公司</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1,722,759</t>
+          <t>800,000</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>USD 90,000</t>
+          <t>$ 355,600</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2 %</t>
+          <t>0 %</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>USD 90,000</t>
+          <t>$ 355,600</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1583,12 +1567,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>資本</t>
+          <t>股票</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Celesta Capital III, L.P.</t>
+          <t>Ayar Labs, Inc.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1598,22 +1582,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,722,759</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>USD 9,883</t>
+          <t>USD 90,000</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2 %</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>USD 9,883</t>
+          <t>USD 90,000</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1635,7 +1619,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Achi Capital Partners Fund LP</t>
+          <t>Celesta Capital III, L.P.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1650,7 +1634,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>USD 74,715</t>
+          <t>USD 9,883</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1660,7 +1644,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>USD 74,715</t>
+          <t>USD 9,883</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1682,12 +1666,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>上海華芯創業投資企業</t>
+          <t>Achi Capital Partners Fund LP</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Gaintech Co. Limited</t>
+          <t>Digimoc Holdings Limited</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1697,7 +1681,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>USD 53,837</t>
+          <t>USD 74,715</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1707,7 +1691,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>USD 53,837</t>
+          <t>USD 74,715</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1729,7 +1713,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Walden Technology Venture II,L.P.</t>
+          <t>上海華芯創業投資企業</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1744,7 +1728,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>USD 11,985</t>
+          <t>USD 53,837</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1754,7 +1738,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>USD 11,985</t>
+          <t>USD 53,837</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1776,7 +1760,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>上海武岳峰集成電路股權投資合夥企業(有限合夥)</t>
+          <t>Walden Technology Venture II,L.P.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1791,7 +1775,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>USD 91,504</t>
+          <t>USD 11,985</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1801,7 +1785,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>USD 91,504</t>
+          <t>USD 11,985</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1823,7 +1807,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>HOPU USD Master Fund III, L.P.</t>
+          <t>上海武岳峰集成電路股權投資合夥企業(有限合夥)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1838,7 +1822,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>USD 31,979</t>
+          <t>USD 91,504</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1848,7 +1832,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>USD 31,979</t>
+          <t>USD 91,504</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1870,7 +1854,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Walden Technology Ventures III, L.P.</t>
+          <t>HOPU USD Master Fund III, L.P.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1885,7 +1869,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>USD 38,532</t>
+          <t>USD 31,979</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1895,7 +1879,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>USD 38,532</t>
+          <t>USD 31,979</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1917,12 +1901,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Prime Movers Growth Fund I L.P.</t>
+          <t>Walden Technology Ventures III, L.P.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>MTKC Global Holdings Co. Limited</t>
+          <t>Gaintech Co. Limited</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1932,7 +1916,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>USD 12,896</t>
+          <t>USD 38,532</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1942,7 +1926,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>USD 12,896</t>
+          <t>USD 38,532</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1964,12 +1948,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>芯愛科技(南京)有限公司</t>
+          <t>Prime Movers Growth Fund I L.P.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>聯發利寶(香港)有限公司</t>
+          <t>MTKC Global Holdings Co. Limited</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1979,7 +1963,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>CNY 90,944</t>
+          <t>USD 12,896</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1989,7 +1973,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>CNY 90,944</t>
+          <t>USD 12,896</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2011,12 +1995,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HEVC ADVANCE LLC</t>
+          <t>芯愛科技(南京)有限公司</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>MediaTek USA Inc.</t>
+          <t>聯發利寶(香港)有限公司</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2026,7 +2010,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>USD 9,517</t>
+          <t>CNY 90,944</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2036,7 +2020,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>USD 9,517</t>
+          <t>CNY 90,944</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2058,12 +2042,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>湖北長江蔚來新能源產業發展基金合伙企業(有限合伙)</t>
+          <t>HEVC ADVANCE LLC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>聯發博動科技(北京)有限公司</t>
+          <t>MediaTek USA Inc.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2073,7 +2057,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>CNY 176,530</t>
+          <t>USD 9,517</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2083,7 +2067,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>CNY 176,530</t>
+          <t>USD 9,517</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2105,12 +2089,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>上海武岳峰二期集成電路股權投資合夥企業(有限合夥)</t>
+          <t>湖北長江蔚來新能源產業發展基金合伙企業(有限合伙)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>聯發軟件設計(深圳)有限公司</t>
+          <t>聯發博動科技(北京)有限公司</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2120,7 +2104,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>CNY 65,234</t>
+          <t>CNY 176,530</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2130,7 +2114,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>CNY 65,234</t>
+          <t>CNY 176,530</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2152,7 +2136,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>南京四維智聯科技有限公司</t>
+          <t>上海武岳峰二期集成電路股權投資合夥企業(有限合夥)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2167,7 +2151,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CNY 368,011</t>
+          <t>CNY 65,234</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2177,7 +2161,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>CNY 368,011</t>
+          <t>CNY 65,234</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2199,162 +2183,146 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
+          <t>南京四維智聯科技有限公司</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>聯發軟件設計(深圳)有限公司</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>CNY 368,011</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>CNY 368,011</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>資本</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
           <t>上海合見工業軟件集團有限公司</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>聯發軟件設計(深圳)有限公司</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
         <is>
           <t>CNY 369,168</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
         <is>
           <t>CNY 369,168</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr">
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
         <is>
           <t>股數</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>帳面金額</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>持股比例</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>持股</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
         <is>
           <t>公允價值</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>資本</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>上海武岳峰浦江二期股權投資合夥企業(有限合夥)</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>聯發科軟件(上海)有限公司</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>CNY 164,300</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>CNY 164,300</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>資本</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>昆橋(深圳)半導體科技產業股權投資基金合夥企業(有限合夥)</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>合肥旭徽聯芯管理諮詢有限公司</t>
-        </is>
-      </c>
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>股數</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>CNY 420,305</t>
+          <t>帳面金額</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>比例</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>CNY 420,305</t>
+          <t>公允價值</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>備註</t>
         </is>
       </c>
     </row>
@@ -2371,12 +2339,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>昆橋二期(廈門)半導體產業股權投資合夥企業(有限合夥)</t>
+          <t>上海武岳峰浦江二期股權投資合夥企業(有限合夥)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>合肥旭徽聯芯管理諮詢有限公司</t>
+          <t>聯發科軟件(上海)有限公司</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2386,7 +2354,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>CNY 304,687</t>
+          <t>CNY 164,300</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2396,7 +2364,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>CNY 304,687</t>
+          <t>CNY 164,300</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2413,17 +2381,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>基金</t>
+          <t>資本</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Fund issued by Cathay Financial Holdings Co., Ltd.</t>
+          <t>昆橋(深圳)半導體科技產業股權投資基金合夥企業(有限合夥)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>合肥旭徽聯芯管理諮詢有限公司</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2433,7 +2401,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>$ 2,008,995</t>
+          <t>CNY 420,305</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2443,7 +2411,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>$ 2,008,995</t>
+          <t>CNY 420,305</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2460,17 +2428,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>基金</t>
+          <t>資本</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Fund issued by Fubon Financial Holding Co., Ltd.</t>
+          <t>昆橋二期(廈門)半導體產業股權投資合夥企業(有限合夥)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>合肥旭徽聯芯管理諮詢有限公司</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2480,7 +2448,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>$ 349,366</t>
+          <t>CNY 304,687</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2490,7 +2458,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>$ 349,366</t>
+          <t>CNY 304,687</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2502,22 +2470,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>按攤銷後成本衡量之金融資產－流動</t>
+          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>債券</t>
+          <t>基金</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>National Bank of Canada</t>
+          <t>Fund issued by Cathay Financial Holdings Co., Ltd.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Hsu Fa (Samoa) Investment Ltd.</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2527,7 +2495,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>CNY 150,000</t>
+          <t>$ 2,008,995</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2537,7 +2505,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>CNY 150,000</t>
+          <t>$ 2,008,995</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2549,22 +2517,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>按攤銷後成本衡量之金融資產－流動</t>
+          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>債券</t>
+          <t>基金</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>JPMorgan Chase &amp; Co.</t>
+          <t>Fund issued by Fubon Financial Holding Co., Ltd.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>旭展(香港)投資有限公司</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2574,7 +2542,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>USD 19,800</t>
+          <t>$ 349,366</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2584,7 +2552,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>USD 20,147</t>
+          <t>$ 349,366</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2606,12 +2574,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Sumitomo Mitsui Banking Corporation</t>
+          <t>National Bank of Canada</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>旭展(香港)投資有限公司</t>
+          <t>Hsu Fa (Samoa) Investment Ltd.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2621,7 +2589,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>USD 13,793</t>
+          <t>CNY 150,000</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2631,7 +2599,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>USD 12,505</t>
+          <t>CNY 150,000</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2653,7 +2621,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Westpac Banking Corporation</t>
+          <t>JPMorgan Chase &amp; Co.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2668,7 +2636,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>USD 23,807</t>
+          <t>USD 19,800</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2678,7 +2646,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>USD 22,696</t>
+          <t>USD 20,147</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2690,7 +2658,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>按攤銷後成本衡量之金融資產－非流動</t>
+          <t>按攤銷後成本衡量之金融資產－流動</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2700,12 +2668,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Fubon Life Insurance Co., Ltd.</t>
+          <t>Sumitomo Mitsui Banking Corporation</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2715,7 +2683,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>$ 490,000</t>
+          <t>USD 13,793</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2725,7 +2693,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>$ 490,309</t>
+          <t>USD 12,505</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2737,7 +2705,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>按攤銷後成本衡量之金融資產－非流動</t>
+          <t>按攤銷後成本衡量之金融資產－流動</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2747,12 +2715,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>KGI Securities Co., Ltd.</t>
+          <t>Westpac Banking Corporation</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2762,7 +2730,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>$ 580,000</t>
+          <t>USD 23,807</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2772,7 +2740,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>$ 576,932</t>
+          <t>USD 22,696</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2794,7 +2762,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
+          <t>Fubon Life Insurance Co., Ltd.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2809,7 +2777,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>$ 400,280</t>
+          <t>$ 490,000</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2819,12 +2787,12 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>$ 398,008</t>
+          <t>$ 490,309</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>註2</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2841,12 +2809,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Bank of America Corporation</t>
+          <t>KGI Securities Co., Ltd.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Hsu Fa (Samoa) Investment Ltd.</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2856,7 +2824,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>CNY 537,000</t>
+          <t>$ 580,000</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2866,7 +2834,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>CNY 545,241</t>
+          <t>$ 576,932</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2888,12 +2856,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Crédit Agricole</t>
+          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Hsu Fa (Samoa) Investment Ltd.</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2903,7 +2871,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>CNY 298,000</t>
+          <t>$ 400,280</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2913,12 +2881,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>CNY 294,579</t>
+          <t>$ 398,008</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>註2</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2903,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>National Bank of Canada</t>
+          <t>Bank of America Corporation</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2950,7 +2918,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>CNY 1,252,000</t>
+          <t>CNY 537,000</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2960,7 +2928,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>CNY 1,274,691</t>
+          <t>CNY 545,241</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2982,7 +2950,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Royal Bank of Canada</t>
+          <t>Crédit Agricole</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2997,7 +2965,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>CNY 561,000</t>
+          <t>CNY 298,000</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3007,7 +2975,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>CNY 561,713</t>
+          <t>CNY 294,579</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3029,7 +2997,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The Goldman Sachs Group, Inc.</t>
+          <t>National Bank of Canada</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3044,7 +3012,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>CNY 395,000</t>
+          <t>CNY 1,252,000</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3054,7 +3022,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>CNY 404,624</t>
+          <t>CNY 1,274,691</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3076,12 +3044,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices, Inc.</t>
+          <t>Royal Bank of Canada</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>旭展(香港)投資有限公司</t>
+          <t>Hsu Fa (Samoa) Investment Ltd.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3091,7 +3059,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>USD 17,147</t>
+          <t>CNY 561,000</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3101,7 +3069,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>USD 16,739</t>
+          <t>CNY 561,713</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3123,12 +3091,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc.</t>
+          <t>The Goldman Sachs Group, Inc.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>旭展(香港)投資有限公司</t>
+          <t>Hsu Fa (Samoa) Investment Ltd.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3138,7 +3106,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>USD 43,198</t>
+          <t>CNY 395,000</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3148,7 +3116,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>USD 41,824</t>
+          <t>CNY 404,624</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3170,7 +3138,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Bank of America Corporation</t>
+          <t>Advanced Micro Devices, Inc.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3185,7 +3153,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>USD 179,007</t>
+          <t>USD 17,147</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3195,7 +3163,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>USD 173,977</t>
+          <t>USD 16,739</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3217,7 +3185,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>BNP Paribas</t>
+          <t>Amazon.com, Inc.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3232,7 +3200,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>USD 44,534</t>
+          <t>USD 43,198</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3242,7 +3210,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>USD 43,829</t>
+          <t>USD 41,824</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3264,7 +3232,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Cathay Life Insurance.</t>
+          <t>Bank of America Corporation</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3279,7 +3247,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>USD 30,000</t>
+          <t>USD 179,007</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3289,7 +3257,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>USD 31,656</t>
+          <t>USD 173,977</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3311,7 +3279,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Citigroup Inc.</t>
+          <t>BNP Paribas</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3326,7 +3294,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>USD 129,515</t>
+          <t>USD 44,534</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3336,7 +3304,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>USD 128,724</t>
+          <t>USD 43,829</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3358,7 +3326,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Crédit Agricole</t>
+          <t>Cathay Life Insurance.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3373,7 +3341,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>USD 37,283</t>
+          <t>USD 30,000</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3383,7 +3351,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>USD 37,285</t>
+          <t>USD 31,656</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3405,7 +3373,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Foxconn Technology Group</t>
+          <t>Citigroup Inc.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3420,7 +3388,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>USD 17,624</t>
+          <t>USD 129,515</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3430,7 +3398,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>USD 17,917</t>
+          <t>USD 128,724</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3452,7 +3420,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>HSBC Holdings plc</t>
+          <t>Crédit Agricole</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3467,7 +3435,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>USD 19,766</t>
+          <t>USD 37,283</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3477,7 +3445,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>USD 19,703</t>
+          <t>USD 37,285</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3499,7 +3467,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ING Group, N.V.</t>
+          <t>Foxconn Technology Group</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3514,7 +3482,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>USD 9,876</t>
+          <t>USD 17,624</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3524,7 +3492,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>USD 9,650</t>
+          <t>USD 17,917</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3546,7 +3514,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>International Business Machines Corporation</t>
+          <t>HSBC Holdings plc</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3561,7 +3529,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>USD 80,261</t>
+          <t>USD 19,766</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3571,7 +3539,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>USD 78,879</t>
+          <t>USD 19,703</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3593,7 +3561,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>JPMorgan Chase &amp; Co.</t>
+          <t>ING Group, N.V.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3608,7 +3576,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>USD 231,613</t>
+          <t>USD 9,876</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3618,7 +3586,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>USD 234,779</t>
+          <t>USD 9,650</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3640,7 +3608,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Mitsubishi UFJ Financial Group, Inc.</t>
+          <t>International Business Machines Corporation</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3655,7 +3623,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>USD 95,579</t>
+          <t>USD 80,261</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3665,7 +3633,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>USD 92,388</t>
+          <t>USD 78,879</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3687,7 +3655,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Mizuho Financial Group, Inc.</t>
+          <t>JPMorgan Chase &amp; Co.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3702,7 +3670,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>USD 140,286</t>
+          <t>USD 231,613</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3712,7 +3680,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>USD 136,672</t>
+          <t>USD 234,779</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3734,7 +3702,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Morgan Stanley</t>
+          <t>Mitsubishi UFJ Financial Group, Inc.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3749,7 +3717,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>USD 255,500</t>
+          <t>USD 95,579</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3759,7 +3727,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>USD 248,385</t>
+          <t>USD 92,388</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3781,7 +3749,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>National Bank of Canada</t>
+          <t>Mizuho Financial Group, Inc.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3796,7 +3764,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>USD 18,000</t>
+          <t>USD 140,286</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3806,7 +3774,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>USD 18,000</t>
+          <t>USD 136,672</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3828,7 +3796,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>NVIDIA CORP</t>
+          <t>Morgan Stanley</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3843,7 +3811,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>USD 24,766</t>
+          <t>USD 255,500</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3853,7 +3821,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>USD 23,288</t>
+          <t>USD 248,385</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3875,7 +3843,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Royal Bank of Canada</t>
+          <t>National Bank of Canada</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3890,7 +3858,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>USD 126,939</t>
+          <t>USD 18,000</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3900,7 +3868,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>USD 127,232</t>
+          <t>USD 18,000</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3922,7 +3890,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Sumitomo Mitsui Banking Corporation</t>
+          <t>NVIDIA CORP</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3937,7 +3905,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>USD 60,279</t>
+          <t>USD 24,766</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3947,7 +3915,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>USD 58,531</t>
+          <t>USD 23,288</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3969,7 +3937,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
+          <t>Royal Bank of Canada</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3984,7 +3952,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>USD 77,898</t>
+          <t>USD 126,939</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3994,7 +3962,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>USD 74,323</t>
+          <t>USD 127,232</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4004,33 +3972,49 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>按攤銷後成本衡量之金融資產－非流動</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>債券</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Sumitomo Mitsui Banking Corporation</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>旭展(香港)投資有限公司</t>
+        </is>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>股數</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>帳面金額</t>
+          <t>USD 60,279</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>持股比例</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>公允價值</t>
+          <t>USD 58,531</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>備註</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4031,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>The Bank of Nova Scotia</t>
+          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4062,7 +4046,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>USD 116,977</t>
+          <t>USD 77,898</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4072,106 +4056,74 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>USD 116,960</t>
+          <t>USD 74,323</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>註2</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>按攤銷後成本衡量之金融資產－非流動</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>債券</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>The Goldman Sachs Group, Inc.</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>旭展(香港)投資有限公司</t>
-        </is>
-      </c>
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>股數</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>USD 77,505</t>
+          <t>帳面金額</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>持股</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>USD 76,752</t>
+          <t>公允價值</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>備註</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>按攤銷後成本衡量之金融資產－非流動</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>債券</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>UBS Group AG</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>旭展(香港)投資有限公司</t>
-        </is>
-      </c>
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>股數</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>USD 9,826</t>
+          <t>帳面金額</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>比例</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>USD 9,888</t>
+          <t>公允價值</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>備註</t>
         </is>
       </c>
     </row>
@@ -4188,35 +4140,176 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
+          <t>The Bank of Nova Scotia</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>旭展(香港)投資有限公司</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>USD 116,977</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>USD 116,960</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>註2</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>按攤銷後成本衡量之金融資產－非流動</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>債券</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>The Goldman Sachs Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>旭展(香港)投資有限公司</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>USD 77,505</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>USD 76,752</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>按攤銷後成本衡量之金融資產－非流動</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>債券</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>UBS Group AG</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>旭展(香港)投資有限公司</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>USD 9,826</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>USD 9,888</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>按攤銷後成本衡量之金融資產－非流動</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>債券</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
           <t>Wells Fargo &amp; Company</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
         <is>
           <t>USD 74,089</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
         <is>
           <t>USD 73,345</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
+      <c r="I85" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
bug fix: more precise pdf_parser & announcement_scraper
</commit_message>
<xml_diff>
--- a/downloads/2454_2026_Q1_重大有價證券.xlsx
+++ b/downloads/2454_2026_Q1_重大有價證券.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,7 +480,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>持股</t>
+          <t>持股 比例</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -495,55 +495,71 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>強制透過損益按公允價值衡量之金融資產－流動</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>組合式商品</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>旭展(香港)投資有限公司</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>股數</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>帳面金額</t>
+          <t>USD 17,737</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>比例</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>公允價值</t>
+          <t>USD 17,737</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>備註</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>強制透過損益按公允價值衡量之金融資產－流動</t>
+          <t>強制透過損益按公允價值衡量之金融資產－非流動</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>組合式商品</t>
+          <t>信託基金</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>JPMorgan Chase &amp; Co.</t>
+          <t>信託基金</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>旭展(香港)投資有限公司</t>
+          <t>MediaTek USA Inc.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -553,7 +569,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>USD 17,737</t>
+          <t>USD 85,438</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -563,7 +579,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>USD 17,737</t>
+          <t>USD 85,438</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -580,17 +596,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>信託基金</t>
+          <t>債券</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>信託基金</t>
+          <t>Carsome Group Convertible Promissory Note</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MediaTek USA Inc.</t>
+          <t>MTKC Global Holdings Co. Limited</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -600,7 +616,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>USD 85,438</t>
+          <t>USD 12,830</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -610,7 +626,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>USD 85,438</t>
+          <t>USD 12,830</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -622,7 +638,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>強制透過損益按公允價值衡量之金融資產－非流動</t>
+          <t>透過其他綜合損益按公允價值衡量之債務工具－流動</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -632,12 +648,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Carsome Group Convertible Promissory Note</t>
+          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MTKC Global Holdings Co. Limited</t>
+          <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -647,7 +663,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>USD 12,830</t>
+          <t>USD 19,810</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -657,7 +673,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>USD 12,830</t>
+          <t>USD 19,810</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -669,42 +685,42 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>透過其他綜合損益按公允價值衡量之債務工具－流動</t>
+          <t>透過其他綜合損益按公允價值衡量之權益工具－流動</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>債券</t>
+          <t>股票</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
+          <t>深圳市匯頂科技股份有限公司</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>旭展(香港)投資有限公司</t>
+          <t>匯發國際(香港)有限公司</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12,476,705</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>USD 19,810</t>
+          <t>USD 114,441</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3 %</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>USD 19,810</t>
+          <t>USD 114,441</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -726,32 +742,32 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>深圳市匯頂科技股份有限公司</t>
+          <t>晶心科技(股)公司</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>匯發國際(香港)有限公司</t>
+          <t>翔發投資(股)公司</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>12,476,705</t>
+          <t>3,249,324</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>USD 114,441</t>
+          <t>$ 558,884</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3 %</t>
+          <t>6 %</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>USD 114,441</t>
+          <t>$ 558,884</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -773,7 +789,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>晶心科技(股)公司</t>
+          <t>中華精測科技(股)公司</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -783,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3,249,324</t>
+          <t>176,000</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>$ 558,884</t>
+          <t>$ 542,080</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>6 %</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>$ 558,884</t>
+          <t>$ 542,080</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -810,7 +826,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>透過其他綜合損益按公允價值衡量之權益工具－流動</t>
+          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -820,32 +836,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>中華精測科技(股)公司</t>
+          <t>富邦金融控股(股)公司乙種特別股</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>翔發投資(股)公司</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>176,000</t>
+          <t>15,000,000</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>$ 542,080</t>
+          <t>$ 937,500</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1 %</t>
+          <t>0 %</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>$ 542,080</t>
+          <t>$ 937,500</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -867,7 +883,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>富邦金融控股(股)公司乙種特別股</t>
+          <t>富邦金融控股(股)公司丙種特別股</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -877,12 +893,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15,000,000</t>
+          <t>7,056,243</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>$ 937,500</t>
+          <t>$ 364,102</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -892,7 +908,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>$ 937,500</t>
+          <t>$ 364,102</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -914,32 +930,32 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>富邦金融控股(股)公司丙種特別股</t>
+          <t>深圳傳音控股股份有限公司</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>Digimoc Holdings Limited</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>7,056,243</t>
+          <t>71,573,109</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>$ 364,102</t>
+          <t>USD 568,139</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>6 %</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>$ 364,102</t>
+          <t>USD 568,139</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -961,7 +977,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>深圳傳音控股股份有限公司</t>
+          <t>AutoX, Inc.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -971,22 +987,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>71,573,109</t>
+          <t>55,009,500</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>USD 568,139</t>
+          <t>USD 80,864</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6 %</t>
+          <t>3 %</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>USD 568,139</t>
+          <t>USD 80,864</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1008,7 +1024,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AutoX, Inc.</t>
+          <t>Aeonsemi, Inc.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1018,22 +1034,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>55,009,500</t>
+          <t>1,417,657</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>USD 80,864</t>
+          <t>USD 18,592</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3 %</t>
+          <t>6 %</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>USD 80,864</t>
+          <t>USD 18,592</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1055,32 +1071,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Aeonsemi, Inc.</t>
+          <t>世芯電子股份有限公司</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Digimoc Holdings Limited</t>
+          <t>聯發資本(股)公司</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1,417,657</t>
+          <t>450,000</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>USD 18,592</t>
+          <t>$ 991,809</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6 %</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>USD 18,592</t>
+          <t>$ 991,809</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1102,32 +1118,32 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>世芯電子股份有限公司</t>
+          <t>ITH Corporation</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>聯發資本(股)公司</t>
+          <t>Gaintech Co. Limited</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>450,000</t>
+          <t>53,889,085</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$ 991,809</t>
+          <t>USD 55,098</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1 %</t>
+          <t>11 %</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$ 991,809</t>
+          <t>USD 55,098</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1149,32 +1165,32 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ITH Corporation</t>
+          <t>TRANSSNET TECHNOLOGY INC.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Gaintech Co. Limited</t>
+          <t>Cloud Ranger Limited</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>53,889,085</t>
+          <t>1,970,316</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>USD 55,098</t>
+          <t>USD 10,730</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>11 %</t>
+          <t>8 %</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>USD 55,098</t>
+          <t>USD 10,730</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1196,7 +1212,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>TRANSSNET TECHNOLOGY INC.</t>
+          <t>Scaleflux Inc.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1206,22 +1222,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1,970,316</t>
+          <t>2,096,587</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>USD 10,730</t>
+          <t>USD 17,475</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>2 %</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>USD 10,730</t>
+          <t>USD 17,475</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1243,32 +1259,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Scaleflux Inc.</t>
+          <t>瀚博半導體(上海)有限公司</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Cloud Ranger Limited</t>
+          <t>MTKC Global Holdings Co. Limited</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2,096,587</t>
+          <t>4,252,861</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>USD 17,475</t>
+          <t>USD 37,420</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2 %</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>USD 17,475</t>
+          <t>USD 37,420</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1290,32 +1306,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>瀚博半導體(上海)有限公司</t>
+          <t>強一半導體(蘇州)有限公司</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>MTKC Global Holdings Co. Limited</t>
+          <t>聯發利寶(香港)有限公司</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>4,252,861</t>
+          <t>2,474,300</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>USD 37,420</t>
+          <t>CNY 586,409</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>1 %</t>
+          <t>2 %</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>USD 37,420</t>
+          <t>CNY 586,409</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1337,32 +1353,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>強一半導體(蘇州)有限公司</t>
+          <t>蘇州思必馳信息科技有限公司</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>聯發利寶(香港)有限公司</t>
+          <t>聯發博動科技(北京)有限公司</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2,474,300</t>
+          <t>4,638,600</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CNY 586,409</t>
+          <t>CNY 75,907</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2 %</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CNY 586,409</t>
+          <t>CNY 75,907</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1384,37 +1400,37 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>蘇州思必馳信息科技有限公司</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>聯發博動科技(北京)有限公司</t>
+          <t>翔發投資(股)公司</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>4,638,600</t>
+          <t>7,794,085</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>CNY 75,907</t>
+          <t>$ 11,613,187</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>1 %</t>
+          <t>0 %</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CNY 75,907</t>
+          <t>$ 11,613,187</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>註1</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1447,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>樺漢科技股份有限公司</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1441,27 +1457,27 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>7,794,085</t>
+          <t>3,682,456</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>$ 11,613,187</t>
+          <t>$ 997,946</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>3 %</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>$ 11,613,187</t>
+          <t>$ 997,946</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>註1</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1478,32 +1494,32 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>樺漢科技股份有限公司</t>
+          <t>欣興電子股份有限公司</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>翔發投資(股)公司</t>
+          <t>聯發資本(股)公司</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>3,682,456</t>
+          <t>800,000</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>$ 997,946</t>
+          <t>$ 355,600</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3 %</t>
+          <t>0 %</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>$ 997,946</t>
+          <t>$ 355,600</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1525,32 +1541,32 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>欣興電子股份有限公司</t>
+          <t>Ayar Labs, Inc.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>聯發資本(股)公司</t>
+          <t>Digimoc Holdings Limited</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>800,000</t>
+          <t>1,722,759</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>$ 355,600</t>
+          <t>USD 90,000</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>2 %</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>$ 355,600</t>
+          <t>USD 90,000</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1567,12 +1583,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>股票</t>
+          <t>資本</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ayar Labs, Inc.</t>
+          <t>Celesta Capital III, L.P.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1582,22 +1598,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1,722,759</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>USD 90,000</t>
+          <t>USD 9,883</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2 %</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>USD 90,000</t>
+          <t>USD 9,883</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1619,7 +1635,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Celesta Capital III, L.P.</t>
+          <t>Achi Capital Partners Fund LP</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1634,7 +1650,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>USD 9,883</t>
+          <t>USD 74,715</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1644,7 +1660,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>USD 9,883</t>
+          <t>USD 74,715</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1666,12 +1682,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Achi Capital Partners Fund LP</t>
+          <t>上海華芯創業投資企業</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Digimoc Holdings Limited</t>
+          <t>Gaintech Co. Limited</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1681,7 +1697,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>USD 74,715</t>
+          <t>USD 53,837</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1691,7 +1707,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>USD 74,715</t>
+          <t>USD 53,837</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1713,7 +1729,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>上海華芯創業投資企業</t>
+          <t>Walden Technology Venture II,L.P.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1728,7 +1744,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>USD 53,837</t>
+          <t>USD 11,985</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1738,7 +1754,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>USD 53,837</t>
+          <t>USD 11,985</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1760,7 +1776,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Walden Technology Venture II,L.P.</t>
+          <t>上海武岳峰集成電路股權投資合夥企業(有限合夥)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1775,7 +1791,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>USD 11,985</t>
+          <t>USD 91,504</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1785,7 +1801,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>USD 11,985</t>
+          <t>USD 91,504</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1807,7 +1823,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>上海武岳峰集成電路股權投資合夥企業(有限合夥)</t>
+          <t>HOPU USD Master Fund III, L.P.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1822,7 +1838,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>USD 91,504</t>
+          <t>USD 31,979</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1832,7 +1848,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>USD 91,504</t>
+          <t>USD 31,979</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1854,7 +1870,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HOPU USD Master Fund III, L.P.</t>
+          <t>Walden Technology Ventures III, L.P.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1869,7 +1885,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>USD 31,979</t>
+          <t>USD 38,532</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1879,7 +1895,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>USD 31,979</t>
+          <t>USD 38,532</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1901,12 +1917,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Walden Technology Ventures III, L.P.</t>
+          <t>Prime Movers Growth Fund I L.P.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Gaintech Co. Limited</t>
+          <t>MTKC Global Holdings Co. Limited</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1916,7 +1932,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>USD 38,532</t>
+          <t>USD 12,896</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1926,7 +1942,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>USD 38,532</t>
+          <t>USD 12,896</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1948,12 +1964,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Prime Movers Growth Fund I L.P.</t>
+          <t>芯愛科技(南京)有限公司</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>MTKC Global Holdings Co. Limited</t>
+          <t>聯發利寶(香港)有限公司</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1963,7 +1979,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>USD 12,896</t>
+          <t>CNY 90,944</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1973,7 +1989,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>USD 12,896</t>
+          <t>CNY 90,944</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1995,12 +2011,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>芯愛科技(南京)有限公司</t>
+          <t>HEVC ADVANCE LLC</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>聯發利寶(香港)有限公司</t>
+          <t>MediaTek USA Inc.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2010,7 +2026,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>CNY 90,944</t>
+          <t>USD 9,517</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2020,7 +2036,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>CNY 90,944</t>
+          <t>USD 9,517</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2042,12 +2058,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HEVC ADVANCE LLC</t>
+          <t>湖北長江蔚來新能源產業發展基金合伙企業(有限合伙)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>MediaTek USA Inc.</t>
+          <t>聯發博動科技(北京)有限公司</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2057,7 +2073,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>USD 9,517</t>
+          <t>CNY 176,530</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2067,7 +2083,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>USD 9,517</t>
+          <t>CNY 176,530</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2089,12 +2105,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>湖北長江蔚來新能源產業發展基金合伙企業(有限合伙)</t>
+          <t>上海武岳峰二期集成電路股權投資合夥企業(有限合夥)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>聯發博動科技(北京)有限公司</t>
+          <t>聯發軟件設計(深圳)有限公司</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2104,7 +2120,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>CNY 176,530</t>
+          <t>CNY 65,234</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2114,7 +2130,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>CNY 176,530</t>
+          <t>CNY 65,234</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2136,7 +2152,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>上海武岳峰二期集成電路股權投資合夥企業(有限合夥)</t>
+          <t>南京四維智聯科技有限公司</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2151,7 +2167,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CNY 65,234</t>
+          <t>CNY 368,011</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2161,7 +2177,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>CNY 65,234</t>
+          <t>CNY 368,011</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2183,7 +2199,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>南京四維智聯科技有限公司</t>
+          <t>上海合見工業軟件集團有限公司</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2198,7 +2214,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CNY 368,011</t>
+          <t>CNY 369,168</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2208,7 +2224,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>CNY 368,011</t>
+          <t>CNY 369,168</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2223,106 +2239,126 @@
           <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>股數</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>帳面金額</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>持股 比例</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>公允價值</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>資本</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>上海合見工業軟件集團有限公司</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>聯發軟件設計(深圳)有限公司</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>CNY 369,168</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>CNY 369,168</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>上海武岳峰浦江二期股權投資合夥企業(有限合夥)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>聯發科軟件(上海)有限公司</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>股數</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>帳面金額</t>
+          <t>CNY 164,300</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>持股</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>公允價值</t>
+          <t>CNY 164,300</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>備註</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>資本</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>昆橋(深圳)半導體科技產業股權投資基金合夥企業(有限合夥)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>合肥旭徽聯芯管理諮詢有限公司</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>股數</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>帳面金額</t>
+          <t>CNY 420,305</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>比例</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>公允價值</t>
+          <t>CNY 420,305</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>備註</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2375,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>上海武岳峰浦江二期股權投資合夥企業(有限合夥)</t>
+          <t>昆橋二期(廈門)半導體產業股權投資合夥企業(有限合夥)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>聯發科軟件(上海)有限公司</t>
+          <t>合肥旭徽聯芯管理諮詢有限公司</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2354,7 +2390,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>CNY 164,300</t>
+          <t>CNY 304,687</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2364,7 +2400,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>CNY 164,300</t>
+          <t>CNY 304,687</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2381,17 +2417,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>資本</t>
+          <t>基金</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>昆橋(深圳)半導體科技產業股權投資基金合夥企業(有限合夥)</t>
+          <t>Fund issued by Cathay Financial Holdings Co., Ltd.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>合肥旭徽聯芯管理諮詢有限公司</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2401,7 +2437,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>CNY 420,305</t>
+          <t>$ 2,008,995</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2411,7 +2447,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>CNY 420,305</t>
+          <t>$ 2,008,995</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2428,17 +2464,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>資本</t>
+          <t>基金</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>昆橋二期(廈門)半導體產業股權投資合夥企業(有限合夥)</t>
+          <t>Fund issued by Fubon Financial Holding Co., Ltd.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>合肥旭徽聯芯管理諮詢有限公司</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2448,7 +2484,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>CNY 304,687</t>
+          <t>$ 349,366</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2458,7 +2494,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>CNY 304,687</t>
+          <t>$ 349,366</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2470,22 +2506,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
+          <t>按攤銷後成本衡量之金融資產－流動</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>基金</t>
+          <t>債券</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Fund issued by Cathay Financial Holdings Co., Ltd.</t>
+          <t>National Bank of Canada</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>Hsu Fa (Samoa) Investment Ltd.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2495,7 +2531,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>$ 2,008,995</t>
+          <t>CNY 150,000</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2505,7 +2541,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>$ 2,008,995</t>
+          <t>CNY 150,000</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2517,22 +2553,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>透過其他綜合損益按公允價值衡量之權益工具－非流動</t>
+          <t>按攤銷後成本衡量之金融資產－流動</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>基金</t>
+          <t>債券</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Fund issued by Fubon Financial Holding Co., Ltd.</t>
+          <t>JPMorgan Chase &amp; Co.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2542,7 +2578,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>$ 349,366</t>
+          <t>USD 19,800</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2552,7 +2588,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>$ 349,366</t>
+          <t>USD 20,147</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2574,12 +2610,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>National Bank of Canada</t>
+          <t>Sumitomo Mitsui Banking Corporation</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Hsu Fa (Samoa) Investment Ltd.</t>
+          <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2589,7 +2625,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>CNY 150,000</t>
+          <t>USD 13,793</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2599,7 +2635,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>CNY 150,000</t>
+          <t>USD 12,505</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2621,7 +2657,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>JPMorgan Chase &amp; Co.</t>
+          <t>Westpac Banking Corporation</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2636,7 +2672,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>USD 19,800</t>
+          <t>USD 23,807</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2646,7 +2682,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>USD 20,147</t>
+          <t>USD 22,696</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2658,7 +2694,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>按攤銷後成本衡量之金融資產－流動</t>
+          <t>按攤銷後成本衡量之金融資產－非流動</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2668,12 +2704,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Sumitomo Mitsui Banking Corporation</t>
+          <t>Fubon Life Insurance Co., Ltd.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>旭展(香港)投資有限公司</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2683,7 +2719,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>USD 13,793</t>
+          <t>$ 490,000</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2693,7 +2729,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>USD 12,505</t>
+          <t>$ 490,309</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2705,7 +2741,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>按攤銷後成本衡量之金融資產－流動</t>
+          <t>按攤銷後成本衡量之金融資產－非流動</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2715,12 +2751,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Westpac Banking Corporation</t>
+          <t>KGI Securities Co., Ltd.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>旭展(香港)投資有限公司</t>
+          <t>聯發科技(股)公司</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2730,7 +2766,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>USD 23,807</t>
+          <t>$ 580,000</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2740,7 +2776,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>USD 22,696</t>
+          <t>$ 576,932</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2762,7 +2798,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Fubon Life Insurance Co., Ltd.</t>
+          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2777,7 +2813,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>$ 490,000</t>
+          <t>$ 400,280</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2787,12 +2823,12 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>$ 490,309</t>
+          <t>$ 398,008</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>註2</t>
         </is>
       </c>
     </row>
@@ -2809,12 +2845,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>KGI Securities Co., Ltd.</t>
+          <t>Bank of America Corporation</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>Hsu Fa (Samoa) Investment Ltd.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2824,7 +2860,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>$ 580,000</t>
+          <t>CNY 537,000</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2834,7 +2870,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>$ 576,932</t>
+          <t>CNY 545,241</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2856,12 +2892,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
+          <t>Crédit Agricole</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>聯發科技(股)公司</t>
+          <t>Hsu Fa (Samoa) Investment Ltd.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2871,7 +2907,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>$ 400,280</t>
+          <t>CNY 298,000</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2881,12 +2917,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>$ 398,008</t>
+          <t>CNY 294,579</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>註2</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2939,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Bank of America Corporation</t>
+          <t>National Bank of Canada</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2918,7 +2954,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>CNY 537,000</t>
+          <t>CNY 1,252,000</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2928,7 +2964,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>CNY 545,241</t>
+          <t>CNY 1,274,691</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2950,7 +2986,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Crédit Agricole</t>
+          <t>Royal Bank of Canada</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2965,7 +3001,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>CNY 298,000</t>
+          <t>CNY 561,000</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2975,7 +3011,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>CNY 294,579</t>
+          <t>CNY 561,713</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2997,7 +3033,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>National Bank of Canada</t>
+          <t>The Goldman Sachs Group, Inc.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3012,7 +3048,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>CNY 1,252,000</t>
+          <t>CNY 395,000</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3022,7 +3058,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>CNY 1,274,691</t>
+          <t>CNY 404,624</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3044,12 +3080,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Royal Bank of Canada</t>
+          <t>Advanced Micro Devices, Inc.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Hsu Fa (Samoa) Investment Ltd.</t>
+          <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3059,7 +3095,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>CNY 561,000</t>
+          <t>USD 17,147</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3069,7 +3105,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>CNY 561,713</t>
+          <t>USD 16,739</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3091,12 +3127,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>The Goldman Sachs Group, Inc.</t>
+          <t>Amazon.com, Inc.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Hsu Fa (Samoa) Investment Ltd.</t>
+          <t>旭展(香港)投資有限公司</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3106,7 +3142,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>CNY 395,000</t>
+          <t>USD 43,198</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3116,7 +3152,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>CNY 404,624</t>
+          <t>USD 41,824</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3138,7 +3174,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices, Inc.</t>
+          <t>Bank of America Corporation</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3153,7 +3189,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>USD 17,147</t>
+          <t>USD 179,007</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3163,7 +3199,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>USD 16,739</t>
+          <t>USD 173,977</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3185,7 +3221,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc.</t>
+          <t>BNP Paribas</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3200,7 +3236,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>USD 43,198</t>
+          <t>USD 44,534</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3210,7 +3246,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>USD 41,824</t>
+          <t>USD 43,829</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3232,7 +3268,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Bank of America Corporation</t>
+          <t>Cathay Life Insurance.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3247,7 +3283,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>USD 179,007</t>
+          <t>USD 30,000</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3257,7 +3293,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>USD 173,977</t>
+          <t>USD 31,656</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3279,7 +3315,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>BNP Paribas</t>
+          <t>Citigroup Inc.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3294,7 +3330,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>USD 44,534</t>
+          <t>USD 129,515</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3304,7 +3340,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>USD 43,829</t>
+          <t>USD 128,724</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3326,7 +3362,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Cathay Life Insurance.</t>
+          <t>Crédit Agricole</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3341,7 +3377,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>USD 30,000</t>
+          <t>USD 37,283</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3351,7 +3387,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>USD 31,656</t>
+          <t>USD 37,285</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3373,7 +3409,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Citigroup Inc.</t>
+          <t>Foxconn Technology Group</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3388,7 +3424,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>USD 129,515</t>
+          <t>USD 17,624</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3398,7 +3434,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>USD 128,724</t>
+          <t>USD 17,917</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3420,7 +3456,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Crédit Agricole</t>
+          <t>HSBC Holdings plc</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3435,7 +3471,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>USD 37,283</t>
+          <t>USD 19,766</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3445,7 +3481,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>USD 37,285</t>
+          <t>USD 19,703</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3467,7 +3503,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Foxconn Technology Group</t>
+          <t>ING Group, N.V.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3482,7 +3518,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>USD 17,624</t>
+          <t>USD 9,876</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3492,7 +3528,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>USD 17,917</t>
+          <t>USD 9,650</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3514,7 +3550,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>HSBC Holdings plc</t>
+          <t>International Business Machines Corporation</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3529,7 +3565,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>USD 19,766</t>
+          <t>USD 80,261</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3539,7 +3575,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>USD 19,703</t>
+          <t>USD 78,879</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3561,7 +3597,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ING Group, N.V.</t>
+          <t>JPMorgan Chase &amp; Co.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3576,7 +3612,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>USD 9,876</t>
+          <t>USD 231,613</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3586,7 +3622,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>USD 9,650</t>
+          <t>USD 234,779</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3608,7 +3644,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>International Business Machines Corporation</t>
+          <t>Mitsubishi UFJ Financial Group, Inc.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3623,7 +3659,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>USD 80,261</t>
+          <t>USD 95,579</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3633,7 +3669,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>USD 78,879</t>
+          <t>USD 92,388</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3655,7 +3691,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>JPMorgan Chase &amp; Co.</t>
+          <t>Mizuho Financial Group, Inc.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3670,7 +3706,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>USD 231,613</t>
+          <t>USD 140,286</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3680,7 +3716,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>USD 234,779</t>
+          <t>USD 136,672</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3702,7 +3738,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Mitsubishi UFJ Financial Group, Inc.</t>
+          <t>Morgan Stanley</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3717,7 +3753,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>USD 95,579</t>
+          <t>USD 255,500</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3727,7 +3763,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>USD 92,388</t>
+          <t>USD 248,385</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3749,7 +3785,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Mizuho Financial Group, Inc.</t>
+          <t>National Bank of Canada</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3764,7 +3800,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>USD 140,286</t>
+          <t>USD 18,000</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3774,7 +3810,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>USD 136,672</t>
+          <t>USD 18,000</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3796,7 +3832,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Morgan Stanley</t>
+          <t>NVIDIA CORP</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3811,7 +3847,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>USD 255,500</t>
+          <t>USD 24,766</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3821,7 +3857,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>USD 248,385</t>
+          <t>USD 23,288</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3843,7 +3879,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>National Bank of Canada</t>
+          <t>Royal Bank of Canada</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3858,7 +3894,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>USD 18,000</t>
+          <t>USD 126,939</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3868,7 +3904,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>USD 18,000</t>
+          <t>USD 127,232</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3890,7 +3926,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>NVIDIA CORP</t>
+          <t>Sumitomo Mitsui Banking Corporation</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3905,7 +3941,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>USD 24,766</t>
+          <t>USD 60,279</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3915,7 +3951,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>USD 23,288</t>
+          <t>USD 58,531</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3937,7 +3973,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Royal Bank of Canada</t>
+          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3952,7 +3988,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>USD 126,939</t>
+          <t>USD 77,898</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3962,7 +3998,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>USD 127,232</t>
+          <t>USD 74,323</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -3977,44 +4013,32 @@
           <t>按攤銷後成本衡量之金融資產－非流動</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>債券</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Sumitomo Mitsui Banking Corporation</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>旭展(香港)投資有限公司</t>
-        </is>
-      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>股數</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>USD 60,279</t>
+          <t>帳面金額</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>持股 比例</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>USD 58,531</t>
+          <t>公允價值</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>備註</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4055,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Co., Ltd.</t>
+          <t>The Bank of Nova Scotia</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4046,7 +4070,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>USD 77,898</t>
+          <t>USD 116,977</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4056,74 +4080,106 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>USD 74,323</t>
+          <t>USD 116,960</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>註2</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>按攤銷後成本衡量之金融資產－非流動</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>債券</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>The Goldman Sachs Group, Inc.</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>旭展(香港)投資有限公司</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>股數</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>帳面金額</t>
+          <t>USD 77,505</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>持股</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>公允價值</t>
+          <t>USD 76,752</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>備註</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>按攤銷後成本衡量之金融資產－非流動</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>債券</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>UBS Group AG</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>旭展(香港)投資有限公司</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>股數</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>帳面金額</t>
+          <t>USD 9,826</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>比例</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>公允價值</t>
+          <t>USD 9,888</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>備註</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4196,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The Bank of Nova Scotia</t>
+          <t>Wells Fargo &amp; Company</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4155,7 +4211,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>USD 116,977</t>
+          <t>USD 74,089</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4165,151 +4221,10 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>USD 116,960</t>
+          <t>USD 73,345</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
-        <is>
-          <t>註2</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>按攤銷後成本衡量之金融資產－非流動</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>債券</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>The Goldman Sachs Group, Inc.</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>旭展(香港)投資有限公司</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>USD 77,505</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>USD 76,752</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>按攤銷後成本衡量之金融資產－非流動</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>債券</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>UBS Group AG</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>旭展(香港)投資有限公司</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>USD 9,826</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>USD 9,888</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>按攤銷後成本衡量之金融資產－非流動</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>債券</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Wells Fargo &amp; Company</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>旭展(香港)投資有限公司</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>USD 74,089</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>USD 73,345</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>